<commit_message>
SI Phase B/C: 4 SOPs (Creator eval, trend decision, competitor analysis, social action) + PMO social Excel Sheet5/6
</commit_message>
<xml_diff>
--- a/PMO/业务协作_社媒团队/社媒团队协作表.xlsx
+++ b/PMO/业务协作_社媒团队/社媒团队协作表.xlsx
@@ -11,6 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2.KOL关注池" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.竞品社媒账号" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.周报接收人" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5.Creator评估表" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6.趋势监测配置" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -65,7 +67,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -75,6 +77,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2280,4 +2285,585 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Creator账号</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>平台</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>粉丝数</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>孩子年龄</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>互动率达标</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>红旗</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>AI合作结论</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>优先级</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>业务确认</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Allison Tolman / New Little Life</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>5万+</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>N/A (IBCLC)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>建议合作：母婴泵奶专家背书，Pitch 首选</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Allison Banfield / Pumping Milk</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>YouTube+Blog</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>1万+</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>0-18个月</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>建议合作：全系列测评，可直接建联</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Jessica Anderson / Genuine Lactation</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Instagram+FB</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>5万+</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>N/A (IBCLC)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>建议合作：可穿戴泵专业</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Tamari Jacob / @onewiththepump</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>1.69万</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>6-18个月</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>中-高</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>建议跟进：排奶教育内容</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>maxinesanz</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>未知</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>0-12个月</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>建议观察：已主动测评 Momcozy</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr"/>
+      <c r="B7" s="2" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr"/>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>监测维度</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>AI推荐监测内容</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>平台</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>监测理由</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>优先级</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>业务确认</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>补充/修改</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>目标 Hashtag</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>#exclusivelypumping / #pumpingmom / #breastpump / #wearablepump / #momcozy</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>TikTok/IG</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>S1/S3 核心品类话题</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr"/>
+      <c r="G2" s="3" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>竞品 Hashtag</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>#elviepump / #willowpump / #spectrababyusa / #eufybaby / #elvie</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>S2 竞品内容监控</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>目标 Subreddit</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>r/breastfeeding / r/exclusivelypumping / r/beyondthebump / r/NewParents</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Reddit</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>S1 用户讨论重点</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr"/>
+      <c r="G4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Facebook Groups</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>社媒团队提供目标公开群组名称和 URL（Sheet 1 已有候选 5 个）</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>S1 FB Groups 监测盲区补充</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>品类关键词</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>wearable pump / hands-free pump / pumping at work / flange size / milk supply</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>S1 用户痛点捕捉</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr"/>
+      <c r="G6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>趋势预警阈值</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>视频数 5K→20K 为增长窗口（增速 &gt;3x/周 触发预警）</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>S3 趋势早期识别</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr"/>
+      <c r="G7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="3" t="inlineStr"/>
+      <c r="G8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr"/>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr"/>
+      <c r="G9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="3" t="inlineStr"/>
+      <c r="G10" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>